<commit_message>
Aggiunge fallback su Ticker per strumenti senza ISIN (crypto) nell'import Excel
</commit_message>
<xml_diff>
--- a/public/template-transazioni.xlsx
+++ b/public/template-transazioni.xlsx
@@ -413,17 +413,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -439,30 +440,35 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Operazione</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Quantità</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Prezzo unitario</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Commissione</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Tassa trattenuta</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Contenitore</t>
         </is>
@@ -479,24 +485,60 @@
           <t>IE00B579F325</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
         <is>
           <t>Acquisto</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>0.064599</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>387</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>PAC ETF</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>USDC</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Acquisto</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>25</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>PAC ETF</t>
         </is>

</xml_diff>